<commit_message>
Apply AHCCCS dispute parameter to Mercy Care Advantage
Sets the Mercy Care Advantage dispute window to 12 months from the date
of service, matching Mercy Care Medicaid and the other AHCCCS plans, at
the practice's direction.

The published January 2026 Advantage manual takes the opposite position
- it states contracted providers have no claim dispute rights on the
product and routes disputed claims back through resubmission - so the
row is marked 'Verify vs manual' and both the limit text and the notes
column carry that conflict, with a prompt to confirm the route with
Mercy Care before filing a dispute rather than a resubmission.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013zbDV9Ht7empPzzJp2fP1n
</commit_message>
<xml_diff>
--- a/Carrier_Timely_Filing_Reference.xlsx
+++ b/Carrier_Timely_Filing_Reference.xlsx
@@ -523,7 +523,7 @@
     <t xml:space="preserve">Resubmission is the only route - contracted providers have no claim dispute rights on this product. Mark the claim "Attention: Resubmissions" so it is not denied as a duplicate. The Advantage manual publishes no separate window, so the AHCCCS resubmission parameter of 12 months from the date of service is applied here</t>
   </si>
   <si>
-    <t xml:space="preserve">None - contracted providers have no claim dispute rights on this product. Federal regulation bars Mercy Care from handling contracted provider complaints through the Medicare Advantage appeals process, so a disputed claim goes back through resubmission</t>
+    <t xml:space="preserve">12 months from the date of service, applied from the AHCCCS parameter at the practice's direction. The published Advantage manual takes the opposite position - it states that contracted providers have no claim dispute rights on this product and directs a disputed claim back through resubmission - so confirm the route with Mercy Care before filing a dispute rather than a resubmission</t>
   </si>
   <si>
     <t xml:space="preserve">Mercy Care Advantage Provider Manual, January 2026 (mercycareaz.org/providers/provider-manual.html)</t>
@@ -532,7 +532,7 @@
     <t xml:space="preserve">Mercy Care Health Plan Advantage (AHCCCS)</t>
   </si>
   <si>
-    <t xml:space="preserve">New claims must be filed within 150 days of the date of service or the eligibility posting date, whichever is later - a shorter window than the 365 days Mercy Care Medicaid allows. Contracted providers have no claim dispute rights on this product: federal regulation bars Mercy Care from handling contracted provider complaints through the Medicare Advantage appeals process, so a disputed claim goes back through resubmission instead. The corrected claim window follows the AHCCCS parameter of 12 months from the date of service, the same as Mercy Care Medicaid.</t>
+    <t xml:space="preserve">New claims must be filed within 150 days of the date of service or the eligibility posting date, whichever is later - a shorter window than the 365 days Mercy Care Medicaid allows. Corrected claim and dispute windows follow the AHCCCS parameter of 12 months from the date of service, the same as Mercy Care Medicaid, applied at the practice's direction. Be aware the published Advantage manual says contracted providers have no claim dispute rights here and routes disputed claims through resubmission instead, so a dispute may be refused on that basis.</t>
   </si>
   <si>
     <t xml:space="preserve">MERCY CARE MEDICAID</t>
@@ -910,7 +910,7 @@
     <t xml:space="preserve">Corrected claims counted from the date of service: AHCCCS, Ambetter, Amerigroup, AZ Complete, Banner University MA, Banner University Medicaid, Cigna, Health Choice Medicaid, Health Choice Pathway, Humana Commercial, Humana MA, Mercy Care Advantage, Mercy Care Medicaid, Oscar Health and Tricare East. On these the original filing clock never restarts, so a slow first pass eats the correction window. Amerigroup, Humana and Mercy Care Advantage fall here by way of the contract or resubmission route rather than a published corrected claim rule.</t>
   </si>
   <si>
-    <t xml:space="preserve">Appeals counted from the date of service: AHCCCS, AZ Complete, Banner University MA, Banner University Medicaid, Health Choice Medicaid and Mercy Care Medicaid - the AHCCCS plans, which allow 12 months from the date of service with a 60 day fallback from the adverse action date on the remittance advice when the denial lands late in that window. Every other appeal window on this list runs from the processed date.</t>
+    <t xml:space="preserve">Appeals counted from the date of service: AHCCCS, AZ Complete, Banner University MA, Banner University Medicaid, Health Choice Medicaid, Mercy Care Advantage and Mercy Care Medicaid - the AHCCCS plans, which allow 12 months from the date of service with a 60 day fallback from the adverse action date on the remittance advice when the denial lands late in that window. Every other appeal window on this list runs from the processed date.</t>
   </si>
   <si>
     <t xml:space="preserve">Traps worth knowing</t>
@@ -943,7 +943,7 @@
     <t xml:space="preserve">UnitedHealthcare allows 180 calendar days from the original remittance date to correct a claim, but that window is capped by the filing limit in the agreement counted from the date of service - whichever closes first governs. On the 90 day UHC products that cap usually bites well before the 180 days does. Include every originally billed line on the correction, not just the line being fixed, or the omitted services are recovered as an overpayment.</t>
   </si>
   <si>
-    <t xml:space="preserve">Mercy Care Advantage gives contracted providers no claim dispute rights at all. Federal regulation bars Mercy Care from running contracted provider complaints through the Medicare Advantage appeals process, so the only route is to resubmit, marked "Attention: Resubmissions". Its 150 day initial limit is also far shorter than the 365 days Mercy Care Medicaid allows - the two products should never be worked the same way.</t>
+    <t xml:space="preserve">Mercy Care Advantage carries the AHCCCS windows on this sheet - 12 months from the date of service to correct and to dispute - at the practice's direction, but its published manual takes the opposite position on disputes: it states that contracted providers have no claim dispute rights on the product, because federal regulation bars Mercy Care from running contracted provider complaints through the Medicare Advantage appeals process, and routes disputed claims back through resubmission marked "Attention: Resubmissions". Confirm the route with Mercy Care before filing a dispute. Its 150 day initial limit is also far shorter than the 365 days Mercy Care Medicaid allows, so the two products should never be worked the same way.</t>
   </si>
   <si>
     <t xml:space="preserve">AHCCCS runs two clocks. The initial claim has to be received within 6 months of the date of service or it is denied outright, but once it has landed inside that window there are 12 months from the date of service to correct it to clean claim status. Missing the first clock cannot be repaired by the second.</t>
@@ -2792,15 +2792,17 @@
       <c r="I27" s="11" t="s">
         <v>50</v>
       </c>
-      <c r="J27" s="9" t="s">
+      <c r="J27" s="11" t="s">
         <v>165</v>
       </c>
-      <c r="K27" s="7"/>
+      <c r="K27" s="7" t="n">
+        <v>365</v>
+      </c>
       <c r="L27" s="9" t="s">
-        <v>20</v>
-      </c>
-      <c r="M27" s="10" t="s">
-        <v>24</v>
+        <v>42</v>
+      </c>
+      <c r="M27" s="11" t="s">
+        <v>50</v>
       </c>
       <c r="N27" s="9" t="s">
         <v>166</v>
@@ -3689,7 +3691,7 @@
       </c>
       <c r="B33" s="24" t="n">
         <f aca="false">COUNTIF('Timely Filing'!$M$5:$M$40,"Confirmed")</f>
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3698,7 +3700,7 @@
       </c>
       <c r="B34" s="24" t="n">
         <f aca="false">COUNTIF('Timely Filing'!$M$5:$M$40,"Verify vs contract")+COUNTIF('Timely Filing'!$M$5:$M$40,"Verify vs manual")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -3716,7 +3718,7 @@
       </c>
       <c r="B36" s="24" t="n">
         <f aca="false">COUNTIF('Timely Filing'!$L$5:$L$40,"Date of service")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>